<commit_message>
booking: spell out concrete UI steps for FE/UI cases in TestCases.xlsx (screen, URL, navigation, on-screen check)
</commit_message>
<xml_diff>
--- a/testcases/TestCases.xlsx
+++ b/testcases/TestCases.xlsx
@@ -8254,7 +8254,9 @@
       </c>
       <c r="G150" s="3" t="inlineStr">
         <is>
-          <t>Then the home page lists the active hotels, once each</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page lists the active hotels, once each.</t>
         </is>
       </c>
       <c r="H150" s="3" t="inlineStr">
@@ -8304,7 +8306,9 @@
       </c>
       <c r="G151" s="3" t="inlineStr">
         <is>
-          <t>Then the home page does not list the inactive hotel</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page does not list the inactive hotel.</t>
         </is>
       </c>
       <c r="H151" s="3" t="inlineStr">
@@ -8354,7 +8358,9 @@
       </c>
       <c r="G152" s="3" t="inlineStr">
         <is>
-          <t>Then every hotel row shows a three-letter currency code</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: every hotel row shows a three-letter currency code.</t>
         </is>
       </c>
       <c r="H152" s="3" t="inlineStr">
@@ -8404,7 +8410,9 @@
       </c>
       <c r="G153" s="3" t="inlineStr">
         <is>
-          <t>Then the home page shows at least one hotel</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. On screen, verify: the home page shows at least one hotel.</t>
         </is>
       </c>
       <c r="H153" s="3" t="inlineStr">
@@ -8454,8 +8462,10 @@
       </c>
       <c r="G154" s="3" t="inlineStr">
         <is>
-          <t>When the hotel page for hotel 1 is opened
-Then every room name on screen equals the room row</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Hotel' screen in the browser (URL /hotel/1) — on Home, click hotel 1.
+4. On screen, verify: every room name on screen equals the room row.</t>
         </is>
       </c>
       <c r="H154" s="3" t="inlineStr">
@@ -8505,8 +8515,10 @@
       </c>
       <c r="G155" s="3" t="inlineStr">
         <is>
-          <t>When the hotel page for hotel 1 is opened
-Then every room rate on screen equals the room row in the hotel's currency</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Hotel' screen in the browser (URL /hotel/1) — on Home, click hotel 1.
+4. On screen, verify: every room rate on screen equals the room row in the hotel's currency.</t>
         </is>
       </c>
       <c r="H155" s="3" t="inlineStr">
@@ -8556,8 +8568,10 @@
       </c>
       <c r="G156" s="3" t="inlineStr">
         <is>
-          <t>When the hotel page for hotel 2 is opened
-Then every room shows its inventory and cancellation policy from the rows</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Hotel' screen in the browser (URL /hotel/2) — on Home, click hotel 2.
+4. On screen, verify: every room shows its inventory and cancellation policy from the rows.</t>
         </is>
       </c>
       <c r="H156" s="3" t="inlineStr">
@@ -8607,8 +8621,10 @@
       </c>
       <c r="G157" s="3" t="inlineStr">
         <is>
-          <t>When the hotel page for hotel 999 is opened
-Then the page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Hotel' screen in the browser (URL /hotel/999) — on Home, click hotel 999.
+4. On screen, verify: the page reports not found.</t>
         </is>
       </c>
       <c r="H157" s="3" t="inlineStr">
@@ -8658,9 +8674,11 @@
       </c>
       <c r="G158" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-When the booking page is opened
-Then the booking page total equals the stored total</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Open the app 'Booking' screen in the browser (URL /booking/&lt;the held booking&gt;) — click the held booking.
+5. On screen, verify: the booking page total equals the stored total.</t>
         </is>
       </c>
       <c r="H158" s="3" t="inlineStr">
@@ -8710,10 +8728,12 @@
       </c>
       <c r="G159" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-When the booking page is opened
-Then the booking page shows the nights from the row
-And the booking page shows status "held"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Open the app 'Booking' screen in the browser (URL /booking/&lt;the held booking&gt;) — click the held booking.
+5. On screen, verify: the booking page shows the nights from the row.
+6. On screen, verify: the booking page shows status "held".</t>
         </is>
       </c>
       <c r="H159" s="3" t="inlineStr">
@@ -8764,9 +8784,11 @@
       </c>
       <c r="G160" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-When the booking page is opened
-Then the booking page total is shown as a currency amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Open the app 'Booking' screen in the browser (URL /booking/&lt;the held booking&gt;) — click the held booking.
+5. On screen, verify: the booking page total is shown as a currency amount.</t>
         </is>
       </c>
       <c r="H160" s="3" t="inlineStr">
@@ -8816,8 +8838,10 @@
       </c>
       <c r="G161" s="3" t="inlineStr">
         <is>
-          <t>When the booking page for 999999 is opened
-Then the page reports not found</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Booking' screen in the browser (URL /booking/999999) — open booking 999999 from the guest's booking list.
+4. On screen, verify: the page reports not found.</t>
         </is>
       </c>
       <c r="H161" s="3" t="inlineStr">
@@ -8867,10 +8891,12 @@
       </c>
       <c r="G162" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-And the booking reaches &lt;state&gt;
-When the booking page is opened
-Then the booking page shows status "&lt;state&gt;"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Set up (before checking the screen): the booking reaches &lt;state&gt;.
+5. Open the app 'Booking' screen in the browser (URL /booking/&lt;the held booking&gt;) — click the held booking.
+6. On screen, verify: the booking page shows status "&lt;state&gt;".</t>
         </is>
       </c>
       <c r="H162" s="3" t="inlineStr">
@@ -8920,10 +8946,12 @@
       </c>
       <c r="G163" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-And the booking reaches &lt;state&gt;
-When the booking page is opened
-Then the booking page shows status "&lt;state&gt;"</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Set up (before checking the screen): the booking reaches &lt;state&gt;.
+5. Open the app 'Booking' screen in the browser (URL /booking/&lt;the held booking&gt;) — click the held booking.
+6. On screen, verify: the booking page shows status "&lt;state&gt;".</t>
         </is>
       </c>
       <c r="H163" s="3" t="inlineStr">
@@ -8973,9 +9001,11 @@
       </c>
       <c r="G164" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-When the guest's booking list is opened
-Then the guest's booking list includes the held booking</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Open the app 'Guest booking list' screen in the browser (URL /guest/&lt;id&gt;/bookings) — open 'My bookings'.
+5. On screen, verify: the guest's booking list includes the held booking.</t>
         </is>
       </c>
       <c r="H164" s="3" t="inlineStr">
@@ -9025,9 +9055,11 @@
       </c>
       <c r="G165" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-When the guest's booking list is opened
-Then each booking row links to its booking page</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Open the app 'Guest booking list' screen in the browser (URL /guest/&lt;id&gt;/bookings) — open 'My bookings'.
+5. On screen, verify: each booking row links to its booking page.</t>
         </is>
       </c>
       <c r="H165" s="3" t="inlineStr">
@@ -9077,9 +9109,11 @@
       </c>
       <c r="G166" s="3" t="inlineStr">
         <is>
-          <t>Given a held booking
-When the guest's booking list is opened
-Then every booking row total is a currency amount</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a held booking.
+4. Open the app 'Guest booking list' screen in the browser (URL /guest/&lt;id&gt;/bookings) — open 'My bookings'.
+5. On screen, verify: every booking row total is a currency amount.</t>
         </is>
       </c>
       <c r="H166" s="3" t="inlineStr">
@@ -9129,8 +9163,10 @@
       </c>
       <c r="G167" s="3" t="inlineStr">
         <is>
-          <t>When the admin page is opened
-Then the admin payment is shown as a number</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+4. On screen, verify: the admin payment is shown as a number.</t>
         </is>
       </c>
       <c r="H167" s="3" t="inlineStr">
@@ -9180,8 +9216,10 @@
       </c>
       <c r="G168" s="3" t="inlineStr">
         <is>
-          <t>When the admin page is opened
-Then every admin status count is a non-negative integer</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+4. On screen, verify: every admin status count is a non-negative integer.</t>
         </is>
       </c>
       <c r="H168" s="3" t="inlineStr">
@@ -9231,9 +9269,11 @@
       </c>
       <c r="G169" s="3" t="inlineStr">
         <is>
-          <t>Given a confirmed booking
-When the admin page is opened
-Then the admin counts include a confirmed booking</t>
+          <t>1. Precondition: the app and its backend service are up and seeded.
+2. Open the app 'Home – hotels' screen in the browser (URL /) — the app landing page.
+3. Set up (before checking the screen): a confirmed booking.
+4. Open the app 'Admin overview' screen in the browser (URL /admin) — on Home, click 'Admin'.
+5. On screen, verify: the admin counts include a confirmed booking.</t>
         </is>
       </c>
       <c r="H169" s="3" t="inlineStr">

</xml_diff>